<commit_message>
Refresh the drifted paper copy, and make drift checkable
The papers here are copies. Canon changed yesterday and this repository did
not, which is a fork with no process behind it. One file had drifted: the
charge paper picked up a scope note in canon saying what its protection
claim covers - that the winding cannot CHANGE while its cycle exists, not
that the cycle persists. The distinction is load-bearing for the CCC
contrast-zero argument, and it was missing here.

tools/check_paper_sync.py reports drift across all 18 copies and refreshes on
request, keeping each copy's local title block and replacing the body, so the
header cleanup is never undone by a refresh. All 18 verified against canon.

SUB_01 carries the same scope, and states the consequence plainly: in this
account charge is a property of a live loop around a thing, not of the thing
alone.

Workbook regenerated so it reflects the updated page.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_Streamlined_Theory.xlsx
+++ b/ED_Streamlined_Theory.xlsx
@@ -3497,7 +3497,7 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>The field is withheld. At the discrete layer ED gets the integral Gauss law but not a determined local inverse-square field. The paper's own fork says you can have that field only by giving up either orientation-blindness or the arrow, which means leaving ED. | The winding is inert: it couples weakly and does not drive the stability landscape. | The quantization and the loop-independence were confirmed in the certified simulator to machine precision. The argument is structural; the simulation checks it. | The paper is strict that no charge spectrum was fitted. Reproducing the familiar ±1 and ∓⅓ pattern by fitting a topology to those values would violate its own discipline, and is not claimed.</t>
+          <t>The field is withheld. At the discrete layer ED gets the integral Gauss law but not a determined local inverse-square field. The paper's own fork says you can have that field only by giving up either orientation-blindness or the arrow, which means leaving ED. | The winding is inert: it couples weakly and does not drive the stability landscape. | What is protected, and what is not (scope added 2026-09-12). The integer cannot change while the loop that carries it exists. The loop is not itself protected: it is made of live participations, and where participation ceases there is no phase to difference and the number has nothing to be a property of, with nothing uncommitted. `Paper_ED_CCC` §3.6.1 turns on exactly this, using it to clear residual charge at the end of a cosmic aeon. The consequence is worth saying plainly: in this account charge is a property of a live loop around a thing, not of the thing alone. | The quantization and the loop-independence were confirmed in the certified simulator to machine precision. The argument is structural; the simulation checks it. | The paper is strict that no charge spectrum was fitted. Reproducing the familiar ±1 and ∓⅓ pattern by fitting a topology to those values would violate its own discipline, and is not claimed.</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>the protection. Changing the winding would mean uncommitting a polarity</t>
+          <t>the protection. Changing the winding would mean uncommitting a polarity. This protects the number while its loop exists; it does not make the loop permanent</t>
         </is>
       </c>
     </row>

</xml_diff>